<commit_message>
Added append data functionality
</commit_message>
<xml_diff>
--- a/student_results.xlsx
+++ b/student_results.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:H4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -513,6 +513,36 @@
         <v>75.75</v>
       </c>
       <c r="H3" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Karthik</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>90</v>
+      </c>
+      <c r="C4" t="n">
+        <v>85</v>
+      </c>
+      <c r="D4" t="n">
+        <v>80</v>
+      </c>
+      <c r="E4" t="n">
+        <v>90</v>
+      </c>
+      <c r="F4" t="n">
+        <v>345</v>
+      </c>
+      <c r="G4" t="n">
+        <v>86.25</v>
+      </c>
+      <c r="H4" t="inlineStr">
         <is>
           <t>A</t>
         </is>

</xml_diff>

<commit_message>
Added input validation for marks
</commit_message>
<xml_diff>
--- a/student_results.xlsx
+++ b/student_results.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:H5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -545,6 +545,36 @@
       <c r="H4" t="inlineStr">
         <is>
           <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Aalia</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>50</v>
+      </c>
+      <c r="C5" t="n">
+        <v>75</v>
+      </c>
+      <c r="D5" t="n">
+        <v>60</v>
+      </c>
+      <c r="E5" t="n">
+        <v>100</v>
+      </c>
+      <c r="F5" t="n">
+        <v>285</v>
+      </c>
+      <c r="G5" t="n">
+        <v>71.25</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>B</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Added pass fail status
</commit_message>
<xml_diff>
--- a/student_results.xlsx
+++ b/student_results.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:I7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -575,6 +575,76 @@
       <c r="H5" t="inlineStr">
         <is>
           <t>B</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Manav</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>80</v>
+      </c>
+      <c r="C6" t="n">
+        <v>85</v>
+      </c>
+      <c r="D6" t="n">
+        <v>90</v>
+      </c>
+      <c r="E6" t="n">
+        <v>100</v>
+      </c>
+      <c r="F6" t="n">
+        <v>355</v>
+      </c>
+      <c r="G6" t="n">
+        <v>88.75</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Aishwarya</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>80</v>
+      </c>
+      <c r="C7" t="n">
+        <v>20</v>
+      </c>
+      <c r="D7" t="n">
+        <v>75</v>
+      </c>
+      <c r="E7" t="n">
+        <v>60</v>
+      </c>
+      <c r="F7" t="n">
+        <v>235</v>
+      </c>
+      <c r="G7" t="n">
+        <v>58.75</v>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Fail</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Added pass fail status feature
</commit_message>
<xml_diff>
--- a/student_results.xlsx
+++ b/student_results.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I7"/>
+  <dimension ref="A1:I5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -457,194 +457,149 @@
           <t>Grade</t>
         </is>
       </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Dhanush</t>
+          <t>Anjali</t>
         </is>
       </c>
       <c r="B2" t="n">
+        <v>90</v>
+      </c>
+      <c r="C2" t="n">
+        <v>100</v>
+      </c>
+      <c r="D2" t="n">
+        <v>76</v>
+      </c>
+      <c r="E2" t="n">
         <v>80</v>
       </c>
-      <c r="C2" t="n">
-        <v>85</v>
-      </c>
-      <c r="D2" t="n">
-        <v>90</v>
-      </c>
-      <c r="E2" t="n">
-        <v>88</v>
-      </c>
       <c r="F2" t="n">
-        <v>343</v>
+        <v>346</v>
       </c>
       <c r="G2" t="n">
-        <v>85.75</v>
+        <v>86.5</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
           <t>A</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Anajli</t>
+          <t>Dhanush</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="C3" t="n">
-        <v>75</v>
+        <v>100</v>
       </c>
       <c r="D3" t="n">
-        <v>80</v>
+        <v>30</v>
       </c>
       <c r="E3" t="n">
-        <v>78</v>
+        <v>100</v>
       </c>
       <c r="F3" t="n">
-        <v>303</v>
+        <v>310</v>
       </c>
       <c r="G3" t="n">
-        <v>75.75</v>
+        <v>77.5</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
           <t>A</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Fail</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Karthik</t>
+          <t>Payal</t>
         </is>
       </c>
       <c r="B4" t="n">
+        <v>80</v>
+      </c>
+      <c r="C4" t="n">
         <v>90</v>
       </c>
-      <c r="C4" t="n">
-        <v>85</v>
-      </c>
       <c r="D4" t="n">
-        <v>80</v>
+        <v>100</v>
       </c>
       <c r="E4" t="n">
-        <v>90</v>
+        <v>65</v>
       </c>
       <c r="F4" t="n">
-        <v>345</v>
+        <v>335</v>
       </c>
       <c r="G4" t="n">
-        <v>86.25</v>
+        <v>83.75</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
           <t>A</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Aalia</t>
+          <t>Aishwarya</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="C5" t="n">
-        <v>75</v>
+        <v>100</v>
       </c>
       <c r="D5" t="n">
         <v>60</v>
       </c>
       <c r="E5" t="n">
-        <v>100</v>
+        <v>75</v>
       </c>
       <c r="F5" t="n">
-        <v>285</v>
+        <v>335</v>
       </c>
       <c r="G5" t="n">
-        <v>71.25</v>
+        <v>83.75</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>B</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Manav</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
-        <v>80</v>
-      </c>
-      <c r="C6" t="n">
-        <v>85</v>
-      </c>
-      <c r="D6" t="n">
-        <v>90</v>
-      </c>
-      <c r="E6" t="n">
-        <v>100</v>
-      </c>
-      <c r="F6" t="n">
-        <v>355</v>
-      </c>
-      <c r="G6" t="n">
-        <v>88.75</v>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
           <t>A</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr">
+      <c r="I5" t="inlineStr">
         <is>
           <t>Pass</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Aishwarya</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>80</v>
-      </c>
-      <c r="C7" t="n">
-        <v>20</v>
-      </c>
-      <c r="D7" t="n">
-        <v>75</v>
-      </c>
-      <c r="E7" t="n">
-        <v>60</v>
-      </c>
-      <c r="F7" t="n">
-        <v>235</v>
-      </c>
-      <c r="G7" t="n">
-        <v>58.75</v>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>Fail</t>
         </is>
       </c>
     </row>

</xml_diff>